<commit_message>
Correct VIU-05: Delete IS available for Custom roles via kebab (matches spec) — per user screenshot
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/custom-roles-test-cases.xlsx
+++ b/custom-roles-test-cases.xlsx
@@ -489,7 +489,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Verification status: VIU (Verify-in-UI) has BEGUN (pass 1, staging, 2026-07-01). 15 findings logged (10 MATCH / 5 DISCREPANCY) — see the 'VIU Findings Log' tab. 108 test cases now VERIFIED (91 MATCH / 17 DISCREPANCY); remaining cases are UNVERIFIED — VIU pending.</t>
+          <t>Verification status: VIU (Verify-in-UI) has BEGUN (pass 1, staging, 2026-07-01). 15 findings logged (11 MATCH / 4 DISCREPANCY (VIU-05 corrected to MATCH 2026-07-01)) — see the 'VIU Findings Log' tab. 108 test cases now VERIFIED (91 MATCH / 17 DISCREPANCY); remaining cases are UNVERIFIED — VIU pending.</t>
         </is>
       </c>
       <c r="B4" s="2" t="n"/>
@@ -796,22 +796,22 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Edit = inline pencil icon; kebab menu has ONLY 'View Permissions'; NO Delete action for any role (system or custom)</t>
+          <t>Custom roles: kebab (three-dot) menu contains 'View Permissions' + 'Delete'. System roles: kebab has 'View Permissions' only (no Delete). Locked roles (Office, Time Clock): view-only (eye icon). Edit is an inline pencil icon on editable roles.</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>DISCREPANCY (Delete absent; Edit is an icon not a menu item)</t>
+          <t>MATCH</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>actions-menu-system.png, actions-menu-custom.png</t>
+          <t>02-roles-list.png; user screenshot 2026-07-01</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Entire SV-7502 Delete-Role flow appears unimplemented in the UI.</t>
+          <t>Corrected 2026-07-01 per user screenshot — earlier probe had only inspected a System role's kebab and wrongly concluded Delete was absent. Delete IS available for Custom roles, matching spec (SV-7502).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
VIU pass 2 (staging, live admin session): confirm Custom Roles labels/dependency behaviors/kebab; log doubled-path sso/check bug + 2 UX discrepancies
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/custom-roles-test-cases.xlsx
+++ b/custom-roles-test-cases.xlsx
@@ -16,7 +16,7 @@
     <sheet name="Digital Inspections" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'VIU Findings Log'!$A$1:$G$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'VIU Findings Log'!$A$1:$G$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Single Permission'!$A$1:$H$118</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Template Edit'!$A$1:$H$42</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Combination - Representative'!$A$1:$H$11</definedName>
@@ -489,7 +489,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Verification status: VIU (Verify-in-UI) has BEGUN (pass 1, staging, 2026-07-01). 15 findings logged (11 MATCH / 4 DISCREPANCY (VIU-05 corrected to MATCH 2026-07-01)) — see the 'VIU Findings Log' tab. 108 test cases now VERIFIED (91 MATCH / 17 DISCREPANCY); remaining cases are UNVERIFIED — VIU pending.</t>
+          <t>Verification status: VIU (Verify-in-UI) pass 2 complete (staging, live admin session, 2026-07-01). 25 findings logged (17 MATCH / 8 DISCREPANCY) — see the 'VIU Findings Log' tab. Pass 2 confirmed exact Custom Roles labels, the silent CRUD cascade, the 'Enable See Financial Data?' popup, and the kebab-menu variants, and logged 3 build-vs-spec discrepancies (doubled '/api/api/sso/check' path, no unsaved-changes guard on Create Role X-close, and the silent-cascade vs confirmation-popup dependency-UX inconsistency). 108 test cases now VERIFIED (91 MATCH / 17 DISCREPANCY); remaining cases are UNVERIFIED — VIU pending.</t>
         </is>
       </c>
       <c r="B4" s="2" t="n"/>
@@ -589,7 +589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1153,8 +1153,378 @@
       </c>
       <c r="G16" s="3" t="inlineStr"/>
     </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>VIU-16</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Create-role entry point &amp; template picker</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Template selection → Role details → Permission editor → Save</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Button labelled exactly 'Create Custom Role' opens a template picker titled 'Choose a template' (subtext 'Start from a template to pre-fill settings, or skip to start from scratch') listing 11 system templates with 'Skip' and 'Apply' buttons. After Skip/Apply → 'Create Role' form with two sections: 'Basic Details' (Role Name [required], Description) and 'Permissions'.</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>VERIFIED (staging, live admin session, 2026-07-01) — MATCH (exact labels confirmed)</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>VIU pass 2 live admin session 2026-07-01</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Confirms/extends VIU-04 and VIU-08 with the exact picker title, subtext, 11-template count, and Skip/Apply button labels.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>VIU-17</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Permission-tree section headings &amp; controls</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Areas: Work Orders, WO Lines, Schedule, Customers, Invoicing, Timesheets, Page Access, cross-cutting toggles</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Exact headings: 'Work orders' (View / Create &amp; Edit / Delete; 'View mode' segmented control Full View / Tech view; toggles 'Review work orders', 'Pick parts', 'Order parts'); 'Work order lines' (Create &amp; Edit / Delete — NO View); 'Schedule' (View / Create &amp; Edit / Delete); 'Customers' (View / Create &amp; Edit / Delete); 'Invoicing &amp; payments' (View / Create &amp; Edit / 'Delete / Reverse'); 'Timesheets' (View / Create &amp; Edit — NO Delete); 'Page Access' toggles: 'Parts Department', 'Reports', 'Customer portal', 'Settings', 'Billing Portal'; 'Cross-Cutting Toggles': 'See Financial Data', 'View and Manage AP/AR Data', 'View History Logs'. Permission search box present; footer buttons 'Cancel' / 'Create'.</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>VERIFIED (staging, live admin session, 2026-07-01) — MATCH (exact section labels captured)</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>VIU pass 2 live admin session 2026-07-01</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>The edit tier is labelled 'Create &amp; Edit' (not 'Edit'); WO Lines has no independent View; Timesheets has no Delete; there is a permission search box.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>VIU-18</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Invoicing third control label ('Delete / Reverse')</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Invoicing &amp; Payments: View / Edit / Delete</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>The Invoicing &amp; payments third (delete-tier) control is labelled exactly 'Delete / Reverse', not just 'Delete'. Other CRUD sections use plain 'Delete'.</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>VERIFIED (staging, live admin session, 2026-07-01) — DISCREPANCY (label 'Delete / Reverse')</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>VIU pass 2 live admin session 2026-07-01</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>Test cases that reference 'Invoicing Delete' should read the control as 'Delete / Reverse' in the editor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>VIU-19</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>View mode control (Full View / Tech view)</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Tech vs Full; UX only, not access control</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Segmented 'View mode' control under Work orders with options 'Full View' and 'Tech view'.</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>VERIFIED (staging, live admin session, 2026-07-01) — MATCH</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>VIU pass 2 live admin session 2026-07-01</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>Confirms VIU-14 (option labels 'Full View' / 'Tech view').</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>VIU-20</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>CRUD tier cascade is SILENT (no popup)</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>CRUD cascade both directions</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Intra-section CRUD tiers cascade silently with no confirmation popup: enabling 'Create &amp; Edit' auto-enables 'View'; enabling 'Delete' auto-enables View + Create &amp; Edit; turning 'View' OFF force-disables Create &amp; Edit + Delete (View is master). Confirmed on Customers: Delete with all off auto-enables View + Create &amp; Edit + Delete silently.</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>VERIFIED (staging, live admin session, 2026-07-01) — MATCH</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>VIU pass 2 live admin session 2026-07-01</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>Confirms VIU-09/VIU-10; adds that the cascade is silent (no modal) and that View acts as master for its section.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>VIU-21</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Invoicing → See Financial Data confirmation popup (exact text)</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Trigger on enabling Invoicing CRUD while See Financial Data OFF</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Enabling Invoicing 'Create &amp; Edit' or 'Delete / Reverse' while 'See Financial Data' is OFF shows a confirmation popup — title 'Enable See Financial Data?', body 'Invoicing &amp; Payments requires See Financial Data. Enable it to grant this permission?', buttons [Cancel] [Enable]. Enable auto-enables Invoicing View+Create&amp;Edit AND See Financial Data. Cancel changes nothing (permission blocked until dependency accepted).</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>VERIFIED (staging, live admin session, 2026-07-01) — MATCH (exact popup text captured)</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>VIU pass 2 live admin session 2026-07-01</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>Confirms VIU-11 with exact title/body/button text. Cross-Cutting toggles (See Financial Data / View and Manage AP/AR Data / View History Logs) toggle independently — no popup, no mutual auto-enable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>VIU-22</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Kebab (⋮) menu variants</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Row actions: Edit / Delete / View Permissions</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Custom role with 0 users (deletable): kebab has 'View Permissions' and 'Delete' (Delete shown in red). Custom role WITH users (not deletable): kebab has only 'View Permissions' (Delete hidden). System roles: kebab has only 'View Permissions'. Locked system roles (Time Clock, Office): NO kebab at all — view-only eye icon + lock icon.</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>VERIFIED (staging, live admin session, 2026-07-01) — MATCH</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>VIU pass 2 live admin session 2026-07-01</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>Confirms/supersedes VIU-05: Delete IS available for deletable Custom roles, but is hidden for Custom roles that have users assigned. Also confirms VIU-06 (locked roles have no kebab).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>VIU-23</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Doubled '/api' prefix on SSO auth-check (session hydration bug)</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Valid cookie session should hydrate the SPA without bouncing an authenticated user to /login</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Staging auto-auth-check requests '/api/api/sso/check' (doubled '/api' prefix, because the axios baseURL already includes /api) → 404, so a valid cookie session does NOT hydrate the SPA and authenticated users are bounced to /login. Correct path should be '/api/sso/check'.</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>DISCREPANCY (functional bug; severity high — blocks session hydration on staging)</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>VIU pass 2 live admin session 2026-07-01</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>Functional build bug, not a spec-wording issue. UI observation only; no secrets/session data recorded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>VIU-24</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>No unsaved-changes confirmation on Create Role dialog X-close</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Unsaved edits should be protected by a discard/unsaved-changes confirmation</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Closing the Create Role dialog via the X with unsaved permission toggles shows NO unsaved-changes / discard confirmation — the changes are silently dropped.</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>DISCREPANCY (UX; unsaved changes silently discarded)</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>VIU pass 2 live admin session 2026-07-01</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>Contrast with the Cancel/X footer; no guard against accidental data loss.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>VIU-25</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Dependency-UX inconsistency (silent cascade vs confirmation popup)</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Consistent UX for permission 'requires' dependencies</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Two different UX treatments for the same underlying 'requires' pattern: intra-section CRUD dependencies auto-cascade SILENTLY (see VIU-20), but the Invoicing → See Financial Data dependency uses an explicit confirmation popup (see VIU-21).</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>DISCREPANCY (UX inconsistency)</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>VIU pass 2 live admin session 2026-07-01</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>Same 'requires' relationship, two divergent UX patterns.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G16"/>
+  <autoFilter ref="A1:G26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3559,7 +3929,7 @@
       <c r="F43" s="3" t="inlineStr">
         <is>
           <t>1. As admin, follow the admin flow to create the custom role. (Step 1 is a 'Choose a template' dialog with Skip / Apply; the footer save button on the Create Role page is labelled 'Create'.)
-2. With See Financial Data OFF, enable Invoicing &amp; Payments View (or any Invoicing CRUD).
+2. With See Financial Data OFF, enable Invoicing &amp; Payments 'Create &amp; Edit' or 'Delete / Reverse' (View alone does NOT trigger the modal).
 3. Click Confirm.
 4. Repeat and click Cancel instead.</t>
         </is>
@@ -3567,10 +3937,10 @@
       <c r="G43" s="3" t="inlineStr">
         <is>
           <t>Step 1: Create Custom Role dialog opens from a blank/no-access template with all permissions OFF.
-Step 2: Financial confirm modal appears: Modal title: "Enable See Financial Data?" Body: "[Area] requires See Financial Data. Enable it to grant this permission?" Buttons: "Cancel" / "Enable" Confirm auto-enables &amp; applies; Cancel reverts. [Build-vs-spec: spec wording differed — see VIU-11.]
+Step 2: Financial confirm modal appears: Modal title: "Enable See Financial Data?" Body: "Invoicing &amp; Payments requires See Financial Data. Enable it to grant this permission?" Buttons: "Cancel" / "Enable". Enable auto-enables See Financial Data and applies Invoicing View+Create&amp;Edit; Cancel changes nothing. [Build-vs-spec: exact wording confirmed live — see VIU-11 and VIU-21.]
 Step 3: See Financial Data auto-enables and the Invoicing checkbox is applied.
 Step 4: The change reverts; See Financial Data stays OFF and the Invoicing checkbox is not applied.
-Overall: Enabling any Invoicing CRUD while See Financial Data is OFF triggers the financial confirm modal; Confirm auto-enables Financial, Cancel reverts.
+Overall: Enabling Invoicing 'Create &amp; Edit' or 'Delete / Reverse' while See Financial Data is OFF triggers the financial confirm modal ('Enable See Financial Data?'); Enable auto-enables Financial + Invoicing View+Create&amp;Edit, Cancel changes nothing. (View alone does not trigger it.)
 VIU status: Spec: Invoicing financial gate — any CRUD triggers confirm modal if See Financial Data OFF. VERIFIED (staging 2026-07-01) — DISCREPANCY; see VIU-11</t>
         </is>
       </c>
@@ -3672,7 +4042,7 @@
         <is>
           <t>1. As admin, follow the admin flow to create the custom role. (Step 1 is a 'Choose a template' dialog with Skip / Apply; the footer save button on the Create Role page is labelled 'Create'.)
 2. Enable See Financial Data; keep View and Manage AP/AR Data OFF.
-3. Enable Invoicing &amp; Payments Delete.
+3. Enable Invoicing &amp; Payments 'Delete / Reverse' (the delete-tier control in this section is labelled 'Delete / Reverse', not plain 'Delete').
 4. Confirm/enable View and Manage AP/AR Data.</t>
         </is>
       </c>
@@ -3680,7 +4050,7 @@
         <is>
           <t>Step 1: Create Custom Role dialog opens from a blank/no-access template with all permissions OFF.
 Step 2: Financial ON; View and Manage AP/AR Data OFF.
-Step 3: The AP/AR gate is enforced: Invoicing Delete additionally requires View and Manage AP/AR Data (a confirm modal / requirement is shown to enable View and Manage AP/AR Data).
+Step 3: The AP/AR gate is enforced: Invoicing Delete / Reverse additionally requires View and Manage AP/AR Data (a confirm modal / requirement is shown to enable View and Manage AP/AR Data).
 Step 4: View and Manage AP/AR Data enables and Invoicing Delete (with Edit+View cascade) is applied.
 Overall: Invoicing Delete cannot be applied without View and Manage AP/AR Data; the AP/AR gate enforces enabling View and Manage AP/AR Data (in addition to the financial gate).
 VIU status: Spec: Invoicing Delete additionally requires Manage AP/AR (AP/AR gate). UNVERIFIED — VIU pending.</t>
@@ -10862,7 +11232,7 @@
           <t>Step 1: Create Custom Role form opens with every permission toggle OFF by default. Role name accepted.
 Step 2: Parts Dept ON (children enabled). WO Edit cascades WO View ON; WO sub-settings available.
 Step 3: Each Edit cascades its View ON. No Delete enabled anywhere.
-Step 4: Both cascade View ON. Financial confirm modal(s): Modal title: "Enable See Financial Data?" Body: "Invoicing/Part Sales requires See Financial Data. Enable it to grant this permission?" Buttons: "Cancel" / "Enable" — click Enable; See Financial Data ON. [Build-vs-spec: spec wording differed — see VIU-11.]
+Step 4: Both cascade View ON. Financial confirm modal(s): Modal title: "Enable See Financial Data?" Body for Invoicing (confirmed exact): "Invoicing &amp; Payments requires See Financial Data. Enable it to grant this permission?" (the Part Sales modal substitutes its own area name). Buttons: "Cancel" / "Enable" — click Enable; See Financial Data ON. [Build-vs-spec: exact Invoicing wording confirmed live — see VIU-11 and VIU-21.]
 Step 5: Sub-settings, AP/AR, Reports ON. All Delete toggles confirmed OFF.
 Step 6: Role saved with exactly the configured toggles. Staff assignment saved. A role change forces the affected user to be logged out.
 Step 7: Login succeeds; the user sees only navigation permitted by the assigned role.

</xml_diff>

<commit_message>
VIU pass 3 (staging, live per-role as Tech): verify CRUD/page/view-mode/financial gating; log /administration path, empty-role limit, re-login propagation
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/custom-roles-test-cases.xlsx
+++ b/custom-roles-test-cases.xlsx
@@ -16,7 +16,7 @@
     <sheet name="Digital Inspections" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'VIU Findings Log'!$A$1:$G$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'VIU Findings Log'!$A$1:$G$32</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Single Permission'!$A$1:$H$118</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Template Edit'!$A$1:$H$42</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Combination - Representative'!$A$1:$H$11</definedName>
@@ -489,7 +489,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Verification status: VIU (Verify-in-UI) pass 2 complete (staging, live admin session, 2026-07-01). 25 findings logged (17 MATCH / 8 DISCREPANCY) — see the 'VIU Findings Log' tab. Pass 2 confirmed exact Custom Roles labels, the silent CRUD cascade, the 'Enable See Financial Data?' popup, and the kebab-menu variants, and logged 3 build-vs-spec discrepancies (doubled '/api/api/sso/check' path, no unsaved-changes guard on Create Role X-close, and the silent-cascade vs confirmation-popup dependency-UX inconsistency). 108 test cases now VERIFIED (91 MATCH / 17 DISCREPANCY); remaining cases are UNVERIFIED — VIU pending.</t>
+          <t>Verification status: VIU (Verify-in-UI) pass 3 complete — per-role verified as the restricted Tech user (tech@shopview.com) on staging, 2026-07-01. 31 findings logged (21 MATCH / 10 DISCREPANCY) — see the 'VIU Findings Log' tab. Pass 2 (live admin session) confirmed exact Custom Roles labels, the silent CRUD cascade, the 'Enable See Financial Data?' popup, and the kebab-menu variants. Pass 3 logged in AS Tech and verified all 11 per-role gate configs behave PER SPEC: CRUD gating (View-only read-only/no New; +Create&amp;Edit shows New; +Delete per-row delete), page-access nav gating (Reports/Customers/combination exact), Settings routes under '/administration', and view-mode/parts/financial effects carried in the permission wrapper (effects inside the WO detail / invoicing). Discrepancies/limits logged: '/settings' 404s (admin lives at '/administration'), a zero-permission role is not creatable (min 1 permission enforced), and permission changes require the user to re-login + settle. Earlier build-vs-spec discrepancies still stand (doubled '/api/api/sso/check' path, no unsaved-changes guard on Create Role X-close, silent-cascade vs confirmation-popup dependency-UX inconsistency). 108 test cases now VERIFIED (91 MATCH / 17 DISCREPANCY); remaining cases are UNVERIFIED — VIU pending.</t>
         </is>
       </c>
       <c r="B4" s="2" t="n"/>
@@ -589,7 +589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1523,8 +1523,230 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>VIU-26</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Per-role CRUD gating on the restricted Tech user (live login)</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>A role granting WO View only should let the user read Work Orders but not create/edit/delete; adding Create &amp; Edit should expose New/edit; adding Delete should expose per-row delete.</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Logged in AS the restricted 'Tech' user (tech@shopview.com) after assigning each config as admin and re-logging-in as Tech. WO View only: Tech sees ONLY the Work Orders nav; WO list is read-only with NO 'New' button and other modules hidden. WO View + Create &amp; Edit: the 'New' button appears (create/edit enabled), no delete. WO View + Create &amp; Edit + Delete: full WO management including per-row delete. All three behaved PER SPEC.</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>VERIFIED (staging, live per-role Tech session, 2026-07-01) — MATCH</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>staging, live per-role (Tech) session, 2026-07-01</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>Confirms the runtime effect of the CRUD tiers on a real restricted user, complementing the editor-side cascade findings (VIU-09/10/20).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>VIU-27</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Per-role page-access nav gating (Reports / Customers / combination) on Tech</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Page-access toggles and area View permissions should gate the exact nav set the user sees.</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>As Tech: Customers View only → ONLY Customers nav, read-only list, other modules hidden. Page Access Reports ON → Reports nav + report suite visible; OFF → Reports nav hidden (gate is exact). Combination WO View + Customers View + Reports ON → nav = EXACTLY Work Orders, Customers, Reports and nothing else. All behaved PER SPEC.</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>VERIFIED (staging, live per-role Tech session, 2026-07-01) — MATCH</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>staging, live per-role (Tech) session, 2026-07-01</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>Nav is the exact union of granted areas + enabled page-access toggles; no leakage of ungranted modules.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>VIU-28</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Settings/admin routes live under /administration (not /settings)</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Page Access Settings ON should expose the Settings/admin routes (Settings, Staff, Roles &amp; Permissions, Locations, Departments).</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>As Tech with Page Access Settings ON: the settings routes are visible under the Administration area — they are CHILDREN of '/administration' (Settings, Staff, Roles &amp; Permissions, Locations, Departments). Navigating to '/settings' returns a 404 'coffee break' page; the working path is '/administration'.</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>VERIFIED (staging, live per-role Tech session, 2026-07-01) — DISCREPANCY (path drift: spec/docs may say /settings; actual is /administration, and /settings 404s)</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>staging, live per-role (Tech) session, 2026-07-01</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>D1: correct any admin/role-config navigation that says '/settings' to '/administration'. In this suite the test-case JSON already navigates to '/administration/roles-permissions', so no literal '/settings' URL required correcting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>VIU-29</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>View-mode / parts / financial effects carried in wrapper; verified inside WO detail</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>WO View Mode (Tech/Full), WO sub-toggles (Pick parts / Order parts), and See Financial Data should take effect for the assigned user.</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>As Tech: the permission wrapper carries view_mode (tech / woTechViewMode), woPickParts/woOrderParts, and seeFinancialData (true/false) correctly. The visible effects manifest INSIDE the WO detail page (and invoicing for financial), NOT on the WO list: the WO list looks the same in Tech vs Full view; Pick/Order parts actions live inside the WO detail; financial figures/prices are not on the WO list and appear in WO detail / invoicing. All behaved PER SPEC.</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>VERIFIED (staging, live per-role Tech session, 2026-07-01) — MATCH (with verification-location note)</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>staging, live per-role (Tech) session, 2026-07-01</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>D3: verification steps for view-mode, delete, pick/order-parts, and see-financial-data must inspect the WO detail (invoicing for financial), not the WO list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>VIU-30</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Empty (zero-permission) role is not creatable</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>A no-access baseline role could be created with zero permissions to represent a true no-access user.</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>Attempting to create a role with zero permissions is rejected — the API enforces 'At least one permission is required.' A true no-access role is therefore not configurable; the minimal case is a single-permission role (e.g. timesheetsView → Tech lands on own Timesheets with an empty top nav).</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>VERIFIED (staging, live per-role Tech session, 2026-07-01) — DISCREPANCY (design limit: min 1 permission enforced)</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>staging, live per-role (Tech) session, 2026-07-01</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>D2: document as a known constraint; any 'empty role' baseline should use a single-permission minimal role instead. No such empty-role baseline login case exists in this suite, so none required conversion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>VIU-31</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Permission propagation requires re-login + brief settle</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>After reassigning a role to a user, the new permissions should apply to that user.</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>After reassigning a role to the Tech user, the new permissions take effect only after the user logs out and logs back in (fresh login) AND a brief settle. Without a fresh login the prior permission set persists. Behaved as observed on every per-role reassignment.</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>VERIFIED (staging, live per-role Tech session, 2026-07-01) — behavior note</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>staging, live per-role (Tech) session, 2026-07-01</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>D4: added as a precondition/note to per-role (assign-and-login-as-user) cases: 'After assigning the role, log out and log back in as the user (fresh login) so the new permissions load.'</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G26"/>
+  <autoFilter ref="A1:G32"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10777,7 +10999,7 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Logged in as an Administrator with full access. Application is on the Custom Roles &amp; Permissions build (Epic SV-7388, SV-7500 enabled). At least one test staff member exists to receive the role. A second browser/session is available to log in as the test staff user.
+          <t>Logged in as an Administrator with full access. Application is on the Custom Roles &amp; Permissions build (Epic SV-7388, SV-7500 enabled). At least one test staff member exists to receive the role. A second browser/session is available to log in as the test staff user. NOTE (permission propagation): after assigning the role, log out and log back in as the user (fresh login) so the new permissions load; allow a brief settle before verifying.
 Role setup: ON: Work Orders &gt; View; Customers &gt; View; Schedule &gt; View. OFF: everything else — no WO Edit/Delete, no WO Lines, no Customers Edit/Delete, no Schedule Edit/Delete, See Financial Data OFF, Invoicing OFF, Parts Department OFF, Part Sales OFF, Catalog OFF, Vendor OFF, Reports OFF, Timesheets OFF, History Logs OFF, Settings OFF, App Settings OFF, View and Manage AP/AR Data OFF. View Mode = Full (UX only).
 Test data: Test staff user 'frontdesk_qa'. One existing work order, one customer, one schedule entry.
 Permission under test: WO View + Customers View + Schedule View, no create/edit/delete, financials OFF | Original type: Combination | Dependency mode: None</t>
@@ -10836,7 +11058,7 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Logged in as an Administrator with full access. Application is on the Custom Roles &amp; Permissions build (Epic SV-7388, SV-7500 enabled). At least one test staff member exists to receive the role. A second browser/session is available to log in as the test staff user.
+          <t>Logged in as an Administrator with full access. Application is on the Custom Roles &amp; Permissions build (Epic SV-7388, SV-7500 enabled). At least one test staff member exists to receive the role. A second browser/session is available to log in as the test staff user. NOTE (permission propagation): after assigning the role, log out and log back in as the user (fresh login) so the new permissions load; allow a brief settle before verifying.
 Role setup: ON: Schedule &gt; View, Edit, Delete; Work Orders &gt; View; Customers &gt; View. OFF: everything else — WO Edit/Delete, WO Lines, Customers Edit/Delete, See Financial Data, Invoicing, Parts Department, Part Sales, Catalog, Vendor, Reports, Timesheets, History Logs, Settings, App Settings, View and Manage AP/AR Data.
 Test data: Test staff user 'scheduler_qa'. Existing schedule entries, work orders, customers.
 Permission under test: Schedule V/E/D + WO View + Customers View, nothing financial | Original type: Combination | Dependency mode: Cascade: auto-enable lower</t>
@@ -10897,7 +11119,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Logged in as an Administrator with full access. Application is on the Custom Roles &amp; Permissions build (Epic SV-7388, SV-7500 enabled). At least one test staff member exists to receive the role. A second browser/session is available to log in as the test staff user.
+          <t>Logged in as an Administrator with full access. Application is on the Custom Roles &amp; Permissions build (Epic SV-7388, SV-7500 enabled). At least one test staff member exists to receive the role. A second browser/session is available to log in as the test staff user. NOTE (permission propagation): after assigning the role, log out and log back in as the user (fresh login) so the new permissions load; allow a brief settle before verifying.
 Role setup: ON: Work Orders &gt; View; Work Order Lines &gt; View, Edit; WO sub-setting Pick Parts; View Mode = Tech View. OFF: everything else — WO Edit/Delete, WO Lines Delete, Review and Order sub-settings, See Financial Data, Invoicing, Parts Department, Part Sales, Catalog, Vendor, Customers, Schedule, Reports, Timesheets, History Logs, Settings, App Settings, View and Manage AP/AR Data.
 Test data: Test staff user 'jrtech_qa'. Work order with lines to pick parts on.
 Permission under test: WO View + WO Lines Edit + Pick Parts + Tech View, financials OFF | Original type: Combination | Dependency mode: Cascade: auto-enable lower</t>
@@ -10911,7 +11133,7 @@
 4. Enable WO sub-setting Pick Parts; set View Mode = Tech View. Leave Review, Order, WO Lines Delete OFF.
 5. Save the role, then go Administration &gt; Staff &gt; open the test user &gt; assign role 'Junior Tech' &gt; Create.
 6. In a separate browser, log in as the test staff user.
-7. POSITIVE: Confirm the UI presents in Tech View. Open a work order, view lines, edit a line, and pick parts.
+7. POSITIVE: Open a work order and confirm the Tech View presentation INSIDE the WO detail page (the WO list looks the same in Tech vs Full view — the difference is on the WO detail). View lines, edit a line, and use Pick Parts (Pick Parts lives inside the WO detail).
 8. NEGATIVE (aggregate): Attempt to edit the WO header, delete a line, use Review/Order actions; check nav for Invoicing/Customers/Schedule/Reports/Parts and financials.</t>
         </is>
       </c>
@@ -10923,7 +11145,7 @@
 Step 4: Pick Parts ON; View Mode = Tech (UX only). Review/Order remain OFF.
 Step 5: Role saved with exactly the configured toggles. Staff assignment saved. A role change forces the affected user to be logged out.
 Step 6: Login succeeds; the user sees only navigation permitted by the assigned role.
-Step 7: Tech View layout shown. WO viewable, lines editable, Pick Parts action available and works.
+Step 7: Tech View layout shown inside the WO detail page. WO viewable, lines editable, Pick Parts action available inside the WO detail and works. [Verification location per VIU-29: view-mode and pick/order-parts effects manifest in the WO detail, not the WO list.]
 Step 8: WO header not editable, line delete unavailable, Review/Order actions absent. Invoicing, Customers, Schedule, Reports, Parts hidden. No financial figures visible.
 Overall: Junior Tech in Tech View can view WOs, edit lines, and pick parts only. WO Lines Edit cascaded View ON. No header edit, no delete, no financials/other areas.
 VIU status: Spec: SV-7388 WO sub-settings require WO View; CRUD cascade; View Mode UX-only. VERIFIED (staging 2026-07-01) — MATCH; see VIU Findings Log</t>
@@ -10958,7 +11180,7 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Logged in as an Administrator with full access. Application is on the Custom Roles &amp; Permissions build (Epic SV-7388, SV-7500 enabled). At least one test staff member exists to receive the role. A second browser/session is available to log in as the test staff user.
+          <t>Logged in as an Administrator with full access. Application is on the Custom Roles &amp; Permissions build (Epic SV-7388, SV-7500 enabled). At least one test staff member exists to receive the role. A second browser/session is available to log in as the test staff user. NOTE (permission propagation): after assigning the role, log out and log back in as the user (fresh login) so the new permissions load; allow a brief settle before verifying.
 Role setup: ON: Parts Department (parent); Catalog &gt; View, Edit; Vendor &gt; View; Part Sales &gt; View; See Financial Data. OFF: everything else — Catalog Delete, Vendor Edit/Delete, Part Sales Edit/Delete, Work Orders, WO Lines, Customers, Schedule, Invoicing, Reports, Timesheets, History Logs, Settings, App Settings, View and Manage AP/AR Data.
 Test data: Test staff user 'partsclerk_qa'. Existing catalog items, vendors, part-sale records.
 Permission under test: Parts Department ON + Catalog V/E + Vendor V + Part Sales V, See Financial Data ON, no WO/Schedule | Original type: Combination | Dependency mode: Multiple</t>
@@ -11023,7 +11245,7 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Logged in as an Administrator with full access. Application is on the Custom Roles &amp; Permissions build (Epic SV-7388, SV-7500 enabled). At least one test staff member exists to receive the role. A second browser/session is available to log in as the test staff user.
+          <t>Logged in as an Administrator with full access. Application is on the Custom Roles &amp; Permissions build (Epic SV-7388, SV-7500 enabled). At least one test staff member exists to receive the role. A second browser/session is available to log in as the test staff user. NOTE (permission propagation): after assigning the role, log out and log back in as the user (fresh login) so the new permissions load; allow a brief settle before verifying.
 Role setup: ON: Work Orders &gt; View; Invoicing &gt; View, Edit; See Financial Data. OFF: everything else — WO Edit/Delete, WO Lines, Invoicing Delete, View and Manage AP/AR Data, Customers, Schedule, Parts Department, Part Sales, Catalog, Vendor, Reports, Timesheets, History Logs, Settings, App Settings.
 Test data: Test staff user 'cashier_qa'. Work order ready to invoice; open invoice.
 Permission under test: WO View + Invoicing View/Edit + See Financial Data ON, AP/AR OFF, no delete | Original type: Combination | Dependency mode: Financial gate: confirm modal</t>
@@ -11037,7 +11259,7 @@
 4. Confirm Invoicing Delete and View and Manage AP/AR Data remain OFF.
 5. Save the role, then go Administration &gt; Staff &gt; open the test user &gt; assign role 'Cashier' &gt; Create.
 6. In a separate browser, log in as the test staff user.
-7. POSITIVE: Open a work order (view), open Invoicing, create/edit an invoice, view financial totals.
+7. POSITIVE: Open a work order (view), open Invoicing, create/edit an invoice, view financial totals INSIDE the WO detail / invoicing screen (financial figures are not on the WO list).
 8. NEGATIVE (aggregate): Attempt to delete an invoice; look for AP/AR actions; edit a WO; check nav for Customers/Schedule/Parts/Reports/Administration.</t>
         </is>
       </c>
@@ -11049,7 +11271,7 @@
 Step 4: Invoicing View+Edit ON, Delete OFF, View and Manage AP/AR Data OFF, See Financial Data ON.
 Step 5: Role saved with exactly the configured toggles. Staff assignment saved. A role change forces the affected user to be logged out.
 Step 6: Login succeeds; the user sees only navigation permitted by the assigned role.
-Step 7: WO viewable; invoice can be viewed and edited; financial totals displayed.
+Step 7: WO viewable; invoice can be viewed and edited; financial totals displayed inside the WO detail / invoicing screen. [Verification location per VIU-29: See-Financial-Data effects manifest in WO detail / invoicing, not the WO list.]
 Step 8: Invoice delete unavailable; no AP/AR actions; WO not editable; Customers, Schedule, Parts, Reports, Administration hidden.
 Overall: Cashier can view WOs and view/edit invoices with financial data. Invoicing Edit triggered the financial modal (See Financial Data ON) and cascaded View. No delete, no AP/AR, no other areas.
 VIU status: Spec: SV-7388 Invoicing financial gate; CRUD cascade; Invoicing Delete requires AP/AR. VERIFIED (staging 2026-07-01) — DISCREPANCY; see VIU-11</t>
@@ -11084,7 +11306,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Logged in as an Administrator with full access. Application is on the Custom Roles &amp; Permissions build (Epic SV-7388, SV-7500 enabled). At least one test staff member exists to receive the role. A second browser/session is available to log in as the test staff user.
+          <t>Logged in as an Administrator with full access. Application is on the Custom Roles &amp; Permissions build (Epic SV-7388, SV-7500 enabled). At least one test staff member exists to receive the role. A second browser/session is available to log in as the test staff user. NOTE (permission propagation): after assigning the role, log out and log back in as the user (fresh login) so the new permissions load; allow a brief settle before verifying.
 Role setup: ON: Reports (all-or-nothing); See Financial Data; View and Manage AP/AR Data. OFF: everything else — all Work Orders/WO Lines/Customers/Schedule/Invoicing/Parts Department/Part Sales/Catalog/Vendor CRUD, Timesheets, History Logs, Settings, App Settings.
 Test data: Test staff user 'analyst_qa'. Reports with financial figures exist.
 Permission under test: Reports ON + See Financial Data ON + View and Manage AP/AR Data ON, all operational CRUD OFF | Original type: Combination | Dependency mode: None</t>
@@ -11143,7 +11365,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Logged in as an Administrator with full access. Application is on the Custom Roles &amp; Permissions build (Epic SV-7388, SV-7500 enabled). At least one test staff member exists to receive the role. A second browser/session is available to log in as the test staff user.
+          <t>Logged in as an Administrator with full access. Application is on the Custom Roles &amp; Permissions build (Epic SV-7388, SV-7500 enabled). At least one test staff member exists to receive the role. A second browser/session is available to log in as the test staff user. NOTE (permission propagation): after assigning the role, log out and log back in as the user (fresh login) so the new permissions load; allow a brief settle before verifying.
 Role setup: ON: Work Orders &gt; View, Edit; Work Order Lines &gt; View, Edit, Delete; Customers &gt; View, Edit; Schedule &gt; View, Edit; Invoicing &gt; View, Edit; WO sub-settings Review, Pick Parts, Order; See Financial Data. OFF: everything else — WO Delete, Customers Delete, Schedule Delete, Invoicing Delete, View and Manage AP/AR Data, Parts Department, Part Sales, Catalog, Vendor, Reports, Timesheets, History Logs, Settings, App Settings.
 Test data: Test staff user 'svcwriter_qa'. Work order with lines, customer, schedule entry, invoice.
 Permission under test: WO V/E, WO Lines V/E/D, Customers V/E, Schedule V/E, Invoicing V/E, Review/Pick/Order ON, Financial ON, AP/AR OFF | Original type: Combination | Dependency mode: Multiple</t>
@@ -11208,7 +11430,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Logged in as an Administrator with full access. Application is on the Custom Roles &amp; Permissions build (Epic SV-7388, SV-7500 enabled). At least one test staff member exists to receive the role. A second browser/session is available to log in as the test staff user.
+          <t>Logged in as an Administrator with full access. Application is on the Custom Roles &amp; Permissions build (Epic SV-7388, SV-7500 enabled). At least one test staff member exists to receive the role. A second browser/session is available to log in as the test staff user. NOTE (permission propagation): after assigning the role, log out and log back in as the user (fresh login) so the new permissions load; allow a brief settle before verifying.
 Role setup: ON: Work Orders &gt; View, Edit; Work Order Lines &gt; View, Edit; Customers &gt; View, Edit; Schedule &gt; View, Edit; Invoicing &gt; View, Edit; Parts Department (parent); Catalog &gt; View, Edit; Vendor &gt; View, Edit; Part Sales &gt; View, Edit; WO sub-settings Review, Pick Parts, Order; See Financial Data; View and Manage AP/AR Data; Reports. OFF: every Delete (WO, WO Lines, Customers, Schedule, Invoicing, Catalog, Vendor, Part Sales); Timesheets; History Logs; Settings; App Settings.
 Test data: Test staff user 'shopmgr_qa'. Records across all covered areas.
 Permission under test: Broad View+Edit across areas, NO Delete anywhere, See Financial Data ON, View and Manage AP/AR Data ON | Original type: Combination | Dependency mode: Multiple</t>
@@ -11271,7 +11493,7 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Logged in as an Administrator with full access. Application is on the Custom Roles &amp; Permissions build (Epic SV-7388, SV-7500 enabled). At least one test staff member exists to receive the role. A second browser/session is available to log in as the test staff user.
+          <t>Logged in as an Administrator with full access. Application is on the Custom Roles &amp; Permissions build (Epic SV-7388, SV-7500 enabled). At least one test staff member exists to receive the role. A second browser/session is available to log in as the test staff user. NOTE (permission propagation): after assigning the role, log out and log back in as the user (fresh login) so the new permissions load; allow a brief settle before verifying.
 Role setup: ON: Timesheets &gt; View, Edit; Work Orders &gt; View. OFF: everything else — Timesheets Delete, WO Edit/Delete, WO Lines, Customers, Schedule, Invoicing, See Financial Data, Parts Department, Part Sales, Catalog, Vendor, Reports, History Logs, Settings, App Settings, View and Manage AP/AR Data.
 Test data: Test staff user 'timekeeper_qa'. Timesheet entries and a work order.
 Permission under test: Timesheets View/Edit + WO View, financials OFF | Original type: Combination | Dependency mode: Cascade: auto-enable lower</t>
@@ -11330,7 +11552,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Logged in as an Administrator with full access. Application is on the Custom Roles &amp; Permissions build (Epic SV-7388, SV-7500 enabled). At least one test staff member exists to receive the role. A second browser/session is available to log in as the test staff user.
+          <t>Logged in as an Administrator with full access. Application is on the Custom Roles &amp; Permissions build (Epic SV-7388, SV-7500 enabled). At least one test staff member exists to receive the role. A second browser/session is available to log in as the test staff user. NOTE (permission propagation): after assigning the role, log out and log back in as the user (fresh login) so the new permissions load; allow a brief settle before verifying.
 Role setup: ON: Work Orders &gt; View; Invoicing &gt; View; History Logs; Reports; See Financial Data; View and Manage AP/AR Data. OFF: everything else — all Edit/Delete toggles, WO Lines, Customers, Schedule, Parts Department, Part Sales, Catalog, Vendor, Timesheets, Settings, App Settings.
 Test data: Test staff user 'auditor_qa'. Work orders, invoices, history log entries, reports.
 Permission under test: WO View + Invoicing View + History Logs ON + Reports ON + See Financial Data ON, no edits/deletes, AP/AR ON | Original type: Combination | Dependency mode: Financial gate: confirm modal</t>
@@ -11456,7 +11678,7 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Logged in as an Administrator with full access. Application is on the Custom Roles &amp; Permissions build (Epic SV-7388, SV-7500 enabled). At least one test staff member exists to receive the role. A second browser/session is available to log in as the test staff user.
+          <t>Logged in as an Administrator with full access. Application is on the Custom Roles &amp; Permissions build (Epic SV-7388, SV-7500 enabled). At least one test staff member exists to receive the role. A second browser/session is available to log in as the test staff user. NOTE (permission propagation): after assigning the role, log out and log back in as the user (fresh login) so the new permissions load; allow a brief settle before verifying.
 Role setup: Intended: Invoicing &gt; View, Edit only. After resolving the financial gate: See Financial Data ON. OFF: everything else — Invoicing Delete, View and Manage AP/AR Data, Work Orders, WO Lines, Customers, Schedule, Parts Department, Part Sales, Catalog, Vendor, Reports, Timesheets, History Logs, Settings, App Settings.
 Test data: Test staff user 'rnd1_qa'. One open invoice.
 Permission under test: Invoicing View/Edit; See Financial Data enabled via modal; nothing else | Original type: Dependency | Dependency mode: Financial gate: confirm modal</t>
@@ -11515,7 +11737,7 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Logged in as an Administrator with full access. Application is on the Custom Roles &amp; Permissions build (Epic SV-7388, SV-7500 enabled). At least one test staff member exists to receive the role. A second browser/session is available to log in as the test staff user.
+          <t>Logged in as an Administrator with full access. Application is on the Custom Roles &amp; Permissions build (Epic SV-7388, SV-7500 enabled). At least one test staff member exists to receive the role. A second browser/session is available to log in as the test staff user. NOTE (permission propagation): after assigning the role, log out and log back in as the user (fresh login) so the new permissions load; allow a brief settle before verifying.
 Role setup: Intended (invalid): Part Sales &gt; View with Parts Department OFF. Expected resolvable state: Part Sales child is hidden/unsavable while parent OFF. If any usable role saved, it is with Parts Department OFF and NO parts child accessible. OFF: everything else.
 Test data: Test staff user 'rnd2_qa'.
 Permission under test: Attempt Part Sales View with Parts Department OFF (unusable combo) | Original type: Negative | Dependency mode: Parent gate: hide children</t>
@@ -11570,7 +11792,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Logged in as an Administrator with full access. Application is on the Custom Roles &amp; Permissions build (Epic SV-7388, SV-7500 enabled). At least one test staff member exists to receive the role. A second browser/session is available to log in as the test staff user.
+          <t>Logged in as an Administrator with full access. Application is on the Custom Roles &amp; Permissions build (Epic SV-7388, SV-7500 enabled). At least one test staff member exists to receive the role. A second browser/session is available to log in as the test staff user. NOTE (permission propagation): after assigning the role, log out and log back in as the user (fresh login) so the new permissions load; allow a brief settle before verifying.
 Role setup: Intended: Work Orders &gt; Delete only. After cascade: Work Orders &gt; View, Edit, Delete all ON. OFF: everything else — WO Lines, Customers, Schedule, Invoicing, See Financial Data, Parts Department, Part Sales, Catalog, Vendor, Reports, Timesheets, History Logs, Settings, App Settings, View and Manage AP/AR Data.
 Test data: Test staff user 'rnd3_qa'. A deletable work order.
 Permission under test: WO Delete requested → WO View+Edit+Delete saved; nothing else | Original type: Dependency | Dependency mode: Cascade: auto-enable lower</t>
@@ -11583,7 +11805,7 @@
 3. Verify the saved role state before assigning.
 4. Save the role, then go Administration &gt; Staff &gt; open the test user &gt; assign role 'RND WO-Cascade' &gt; Create.
 5. In a separate browser, log in as the test staff user.
-6. POSITIVE: Open Work Orders; view, edit, and delete a work order.
+6. POSITIVE: Open Work Orders; view, edit, and delete a work order. Confirm the delete control (per-row delete on the list and/or inside the WO detail) is present and works.
 7. NEGATIVE (aggregate): Check nav for WO Lines actions, Customers, Schedule, Invoicing, Parts, Reports, Administration; check for financials.</t>
         </is>
       </c>
@@ -11594,7 +11816,7 @@
 Step 3: Saved role has WO View+Edit+Delete ON; no other toggle ON. No financial modal (WO not financial-gated).
 Step 4: Role saved with exactly the configured toggles. Staff assignment saved. A role change forces the affected user to be logged out.
 Step 5: Login succeeds; the user sees only navigation permitted by the assigned role.
-Step 6: All three WO operations succeed (cascade granted View+Edit alongside Delete).
+Step 6: All three WO operations succeed (cascade granted View+Edit alongside Delete); the per-row delete action is available. [Verification location per VIU-29: delete/edit effects are confirmed via the per-row delete and inside the WO detail.]
 Step 7: No WO Lines edit (separate area, not enabled), and all other areas hidden; no financial data shown.
 Overall: Requesting only WO Delete produced a saved role with WO View+Edit+Delete via cascade. User can fully manage WOs; nothing else is accessible.
 VIU status: Spec: SV-7388 CRUD cascade Delete→Edit→View. VERIFIED (staging 2026-07-01) — MATCH; see VIU Findings Log</t>
@@ -11629,7 +11851,7 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Logged in as an Administrator with full access. Application is on the Custom Roles &amp; Permissions build (Epic SV-7388, SV-7500 enabled). At least one test staff member exists to receive the role. A second browser/session is available to log in as the test staff user.
+          <t>Logged in as an Administrator with full access. Application is on the Custom Roles &amp; Permissions build (Epic SV-7388, SV-7500 enabled). At least one test staff member exists to receive the role. A second browser/session is available to log in as the test staff user. NOTE (permission propagation): after assigning the role, log out and log back in as the user (fresh login) so the new permissions load; allow a brief settle before verifying.
 Role setup: ON: Parts Department (parent); Catalog &gt; View, Edit, Delete; Vendor &gt; View, Edit. OFF: everything else — Vendor Delete, Part Sales (all), See Financial Data, Work Orders, WO Lines, Customers, Schedule, Invoicing, Reports, Timesheets, History Logs, Settings, App Settings, View and Manage AP/AR Data.
 Test data: Test staff user 'rnd4_qa'. Catalog items and vendors.
 Permission under test: Parts Dept ON + Catalog V/E/D + Vendor V/E; everything else OFF | Original type: Combination | Dependency mode: Multiple</t>
@@ -11690,7 +11912,7 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Logged in as an Administrator with full access. Application is on the Custom Roles &amp; Permissions build (Epic SV-7388, SV-7500 enabled). At least one test staff member exists to receive the role. A second browser/session is available to log in as the test staff user.
+          <t>Logged in as an Administrator with full access. Application is on the Custom Roles &amp; Permissions build (Epic SV-7388, SV-7500 enabled). At least one test staff member exists to receive the role. A second browser/session is available to log in as the test staff user. NOTE (permission propagation): after assigning the role, log out and log back in as the user (fresh login) so the new permissions load; allow a brief settle before verifying.
 Role setup: ON: Work Orders &gt; View; Schedule &gt; View, Edit; Timesheets &gt; View; Reports; History Logs. OFF: everything else — WO Edit/Delete, WO Lines, Schedule Delete, Timesheets Edit/Delete, Customers, Invoicing, See Financial Data, Parts Department, Part Sales, Catalog, Vendor, Settings, App Settings, View and Manage AP/AR Data.
 Test data: Test staff user 'rnd5_qa'. WOs, schedule entries, timesheets, reports, history entries.
 Permission under test: WO View + Schedule V/E + Timesheets View + Reports ON + History Logs ON, financials OFF | Original type: Combination | Dependency mode: Cascade: auto-enable lower</t>
@@ -11749,7 +11971,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Logged in as an Administrator with full access. Application is on the Custom Roles &amp; Permissions build (Epic SV-7388, SV-7500 enabled). At least one test staff member exists to receive the role. A second browser/session is available to log in as the test staff user.
+          <t>Logged in as an Administrator with full access. Application is on the Custom Roles &amp; Permissions build (Epic SV-7388, SV-7500 enabled). At least one test staff member exists to receive the role. A second browser/session is available to log in as the test staff user. NOTE (permission propagation): after assigning the role, log out and log back in as the user (fresh login) so the new permissions load; allow a brief settle before verifying.
 Role setup: Intended: Invoicing &gt; Delete. After gates resolved: Invoicing View+Edit+Delete ON, See Financial Data ON, View and Manage AP/AR Data ON. OFF: everything else — Work Orders, WO Lines, Customers, Schedule, Parts Department, Part Sales, Catalog, Vendor, Reports, Timesheets, History Logs, Settings, App Settings.
 Test data: Test staff user 'rnd6_qa'. A deletable invoice.
 Permission under test: Invoicing V/E/D requiring See Financial Data + View and Manage AP/AR Data; nothing else | Original type: Dependency | Dependency mode: Multiple</t>
@@ -11810,7 +12032,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Logged in as an Administrator with full access. Application is on the Custom Roles &amp; Permissions build (Epic SV-7388, SV-7500 enabled). At least one test staff member exists to receive the role. A second browser/session is available to log in as the test staff user.
+          <t>Logged in as an Administrator with full access. Application is on the Custom Roles &amp; Permissions build (Epic SV-7388, SV-7500 enabled). At least one test staff member exists to receive the role. A second browser/session is available to log in as the test staff user. NOTE (permission propagation): after assigning the role, log out and log back in as the user (fresh login) so the new permissions load; allow a brief settle before verifying.
 Role setup: ON: Settings; App Settings; Work Orders &gt; View. OFF: everything else — WO Edit/Delete, WO Lines, Customers, Schedule, Invoicing, See Financial Data, Parts Department, Part Sales, Catalog, Vendor, Reports, Timesheets, History Logs, View and Manage AP/AR Data.
 Test data: Test staff user 'rnd7_qa'.
 Permission under test: Settings ON + App Settings ON (enables managing Roles/Staff) + WO View; everything else OFF | Original type: Combination | Dependency mode: Multiple</t>
@@ -11869,7 +12091,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Logged in as an Administrator with full access. Application is on the Custom Roles &amp; Permissions build (Epic SV-7388, SV-7500 enabled). At least one test staff member exists to receive the role. A second browser/session is available to log in as the test staff user.
+          <t>Logged in as an Administrator with full access. Application is on the Custom Roles &amp; Permissions build (Epic SV-7388, SV-7500 enabled). At least one test staff member exists to receive the role. A second browser/session is available to log in as the test staff user. NOTE (permission propagation): after assigning the role, log out and log back in as the user (fresh login) so the new permissions load; allow a brief settle before verifying.
 Role setup: ON: Customers &gt; View, Edit, Delete; Work Order Lines &gt; View, Edit; Parts Department (parent); Vendor &gt; View; View Mode = Full (UX only). OFF: everything else — Work Orders View/Edit/Delete, WO Lines Delete, Catalog (all), Part Sales (all), Vendor Edit/Delete, Schedule, Invoicing, See Financial Data, Reports, Timesheets, History Logs, Settings, App Settings, View and Manage AP/AR Data.
 Test data: Test staff user 'rnd8_qa'. Customers, a work order with lines, vendors.
 Permission under test: Customers V/E/D + WO Lines V/E + Parts Dept ON + Vendor V; Full View mode; financials OFF | Original type: Combination | Dependency mode: Multiple</t>

</xml_diff>